<commit_message>
Small modifications, more disassembly
</commit_message>
<xml_diff>
--- a/Data/Info.xlsx
+++ b/Data/Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52677604-1F6E-46B8-9BFD-35BA113ACBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80900B9A-6604-4D29-9BA8-FBC45DB5CAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="266">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -827,6 +827,21 @@
   </si>
   <si>
     <t>0x3A</t>
+  </si>
+  <si>
+    <t>MSB</t>
+  </si>
+  <si>
+    <t>LSB</t>
+  </si>
+  <si>
+    <t>0x03</t>
+  </si>
+  <si>
+    <t>0x37</t>
+  </si>
+  <si>
+    <t>0xf0</t>
   </si>
 </sst>
 </file>
@@ -1331,9 +1346,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1345,6 +1357,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8624,29 +8639,29 @@
       <c r="AS2" s="64"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>241</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="K3" s="70" t="s">
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="K3" s="69" t="s">
         <v>171</v>
       </c>
-      <c r="L3" s="70"/>
+      <c r="L3" s="69"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="70" t="s">
+      <c r="N3" s="69" t="s">
         <v>172</v>
       </c>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="70"/>
-      <c r="S3" s="70"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="69"/>
+      <c r="R3" s="69"/>
+      <c r="S3" s="69"/>
     </row>
     <row r="4" spans="2:45" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -9122,11 +9137,11 @@
       <c r="S13" s="56">
         <v>0</v>
       </c>
-      <c r="Y13" s="71" t="s">
+      <c r="Y13" s="70" t="s">
         <v>215</v>
       </c>
-      <c r="Z13" s="71"/>
-      <c r="AA13" s="71"/>
+      <c r="Z13" s="70"/>
+      <c r="AA13" s="70"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9135,11 +9150,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="Y14" s="72" t="s">
+      <c r="Y14" s="71" t="s">
         <v>234</v>
       </c>
-      <c r="Z14" s="72"/>
-      <c r="AA14" s="72"/>
+      <c r="Z14" s="71"/>
+      <c r="AA14" s="71"/>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9150,11 +9165,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="Y15" s="73" t="s">
+      <c r="Y15" s="72" t="s">
         <v>235</v>
       </c>
-      <c r="Z15" s="73"/>
-      <c r="AA15" s="73"/>
+      <c r="Z15" s="72"/>
+      <c r="AA15" s="72"/>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9165,40 +9180,40 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="15:45" x14ac:dyDescent="0.25">
-      <c r="O18" s="70" t="s">
+      <c r="O18" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
-      <c r="V18" s="70"/>
-      <c r="W18" s="70"/>
-      <c r="Y18" s="70" t="s">
+      <c r="P18" s="69"/>
+      <c r="Q18" s="69"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="69"/>
+      <c r="U18" s="69"/>
+      <c r="V18" s="69"/>
+      <c r="W18" s="69"/>
+      <c r="Y18" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="Z18" s="70"/>
-      <c r="AA18" s="70"/>
-      <c r="AB18" s="70"/>
-      <c r="AC18" s="70"/>
-      <c r="AD18" s="70"/>
-      <c r="AE18" s="70"/>
-      <c r="AF18" s="70"/>
-      <c r="AG18" s="70"/>
-      <c r="AH18" s="70"/>
-      <c r="AI18" s="70"/>
-      <c r="AJ18" s="70"/>
-      <c r="AK18" s="70"/>
-      <c r="AL18" s="70"/>
-      <c r="AM18" s="70"/>
-      <c r="AN18" s="70"/>
-      <c r="AO18" s="70"/>
-      <c r="AP18" s="70"/>
-      <c r="AQ18" s="70"/>
-      <c r="AR18" s="70"/>
-      <c r="AS18" s="70"/>
+      <c r="Z18" s="69"/>
+      <c r="AA18" s="69"/>
+      <c r="AB18" s="69"/>
+      <c r="AC18" s="69"/>
+      <c r="AD18" s="69"/>
+      <c r="AE18" s="69"/>
+      <c r="AF18" s="69"/>
+      <c r="AG18" s="69"/>
+      <c r="AH18" s="69"/>
+      <c r="AI18" s="69"/>
+      <c r="AJ18" s="69"/>
+      <c r="AK18" s="69"/>
+      <c r="AL18" s="69"/>
+      <c r="AM18" s="69"/>
+      <c r="AN18" s="69"/>
+      <c r="AO18" s="69"/>
+      <c r="AP18" s="69"/>
+      <c r="AQ18" s="69"/>
+      <c r="AR18" s="69"/>
+      <c r="AS18" s="69"/>
     </row>
     <row r="19" spans="15:45" x14ac:dyDescent="0.25">
       <c r="P19" s="46" t="s">
@@ -9368,12 +9383,12 @@
       <c r="U22" s="48" t="s">
         <v>212</v>
       </c>
-      <c r="Y22" s="69" t="s">
+      <c r="Y22" s="73" t="s">
         <v>240</v>
       </c>
-      <c r="Z22" s="69"/>
-      <c r="AA22" s="69"/>
-      <c r="AB22" s="69"/>
+      <c r="Z22" s="73"/>
+      <c r="AA22" s="73"/>
+      <c r="AB22" s="73"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
@@ -10018,16 +10033,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="Y22:AB22"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="O18:W18"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="B2:AS2"/>
     <mergeCell ref="Y18:AS18"/>
     <mergeCell ref="Y13:AA13"/>
     <mergeCell ref="Y14:AA14"/>
     <mergeCell ref="Y15:AA15"/>
-    <mergeCell ref="Y22:AB22"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="O18:W18"/>
-    <mergeCell ref="B3:I3"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10438,43 +10453,70 @@
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
+      <c r="B65" s="58" t="s">
         <v>128</v>
       </c>
+      <c r="D65" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B66" t="s">
+      <c r="B66" s="60" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
+      <c r="B67" s="59" t="s">
         <v>130</v>
+      </c>
+      <c r="D67" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>103</v>
       </c>
+      <c r="E68" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
+      <c r="B69" s="58" t="s">
         <v>104</v>
       </c>
+      <c r="D69" t="s">
+        <v>261</v>
+      </c>
+      <c r="E69" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
+      <c r="B70" s="60" t="s">
         <v>105</v>
       </c>
+      <c r="E70" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B71" t="s">
+      <c r="B71" s="59" t="s">
         <v>106</v>
+      </c>
+      <c r="D71" t="s">
+        <v>262</v>
+      </c>
+      <c r="E71" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>107</v>
+      </c>
+      <c r="E72" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added N30 schema/PCB Small additions to disassembly
</commit_message>
<xml_diff>
--- a/Data/Info.xlsx
+++ b/Data/Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80900B9A-6604-4D29-9BA8-FBC45DB5CAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77490ADA-51A1-4349-9C52-8A9C9B4381CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="N2 (Display)" sheetId="7" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId4"/>
     <sheet name="InternalMemory" sheetId="6" r:id="rId5"/>
+    <sheet name="N30" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'MainBoard-Relais'!$A$1:$AZ$47</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="276">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -842,6 +843,36 @@
   </si>
   <si>
     <t>0xf0</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>something with Galvanic Isolation Card</t>
+  </si>
+  <si>
+    <t>1 = N30.R3019=1, Galvanic type 1</t>
+  </si>
+  <si>
+    <t>Statemachine?</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>/WR</t>
+  </si>
+  <si>
+    <t>READ</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D6</t>
   </si>
 </sst>
 </file>
@@ -1190,7 +1221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1346,6 +1377,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1358,9 +1392,8 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8639,29 +8672,29 @@
       <c r="AS2" s="64"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="70" t="s">
         <v>241</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="K3" s="69" t="s">
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="K3" s="70" t="s">
         <v>171</v>
       </c>
-      <c r="L3" s="69"/>
+      <c r="L3" s="70"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="69" t="s">
+      <c r="N3" s="70" t="s">
         <v>172</v>
       </c>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="70"/>
+      <c r="S3" s="70"/>
     </row>
     <row r="4" spans="2:45" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -9137,11 +9170,11 @@
       <c r="S13" s="56">
         <v>0</v>
       </c>
-      <c r="Y13" s="70" t="s">
+      <c r="Y13" s="71" t="s">
         <v>215</v>
       </c>
-      <c r="Z13" s="70"/>
-      <c r="AA13" s="70"/>
+      <c r="Z13" s="71"/>
+      <c r="AA13" s="71"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9150,11 +9183,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="Y14" s="71" t="s">
+      <c r="Y14" s="72" t="s">
         <v>234</v>
       </c>
-      <c r="Z14" s="71"/>
-      <c r="AA14" s="71"/>
+      <c r="Z14" s="72"/>
+      <c r="AA14" s="72"/>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9165,11 +9198,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="Y15" s="72" t="s">
+      <c r="Y15" s="73" t="s">
         <v>235</v>
       </c>
-      <c r="Z15" s="72"/>
-      <c r="AA15" s="72"/>
+      <c r="Z15" s="73"/>
+      <c r="AA15" s="73"/>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9180,40 +9213,40 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="15:45" x14ac:dyDescent="0.25">
-      <c r="O18" s="69" t="s">
+      <c r="O18" s="70" t="s">
         <v>166</v>
       </c>
-      <c r="P18" s="69"/>
-      <c r="Q18" s="69"/>
-      <c r="R18" s="69"/>
-      <c r="S18" s="69"/>
-      <c r="T18" s="69"/>
-      <c r="U18" s="69"/>
-      <c r="V18" s="69"/>
-      <c r="W18" s="69"/>
-      <c r="Y18" s="69" t="s">
+      <c r="P18" s="70"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="70"/>
+      <c r="S18" s="70"/>
+      <c r="T18" s="70"/>
+      <c r="U18" s="70"/>
+      <c r="V18" s="70"/>
+      <c r="W18" s="70"/>
+      <c r="Y18" s="70" t="s">
         <v>216</v>
       </c>
-      <c r="Z18" s="69"/>
-      <c r="AA18" s="69"/>
-      <c r="AB18" s="69"/>
-      <c r="AC18" s="69"/>
-      <c r="AD18" s="69"/>
-      <c r="AE18" s="69"/>
-      <c r="AF18" s="69"/>
-      <c r="AG18" s="69"/>
-      <c r="AH18" s="69"/>
-      <c r="AI18" s="69"/>
-      <c r="AJ18" s="69"/>
-      <c r="AK18" s="69"/>
-      <c r="AL18" s="69"/>
-      <c r="AM18" s="69"/>
-      <c r="AN18" s="69"/>
-      <c r="AO18" s="69"/>
-      <c r="AP18" s="69"/>
-      <c r="AQ18" s="69"/>
-      <c r="AR18" s="69"/>
-      <c r="AS18" s="69"/>
+      <c r="Z18" s="70"/>
+      <c r="AA18" s="70"/>
+      <c r="AB18" s="70"/>
+      <c r="AC18" s="70"/>
+      <c r="AD18" s="70"/>
+      <c r="AE18" s="70"/>
+      <c r="AF18" s="70"/>
+      <c r="AG18" s="70"/>
+      <c r="AH18" s="70"/>
+      <c r="AI18" s="70"/>
+      <c r="AJ18" s="70"/>
+      <c r="AK18" s="70"/>
+      <c r="AL18" s="70"/>
+      <c r="AM18" s="70"/>
+      <c r="AN18" s="70"/>
+      <c r="AO18" s="70"/>
+      <c r="AP18" s="70"/>
+      <c r="AQ18" s="70"/>
+      <c r="AR18" s="70"/>
+      <c r="AS18" s="70"/>
     </row>
     <row r="19" spans="15:45" x14ac:dyDescent="0.25">
       <c r="P19" s="46" t="s">
@@ -9383,12 +9416,12 @@
       <c r="U22" s="48" t="s">
         <v>212</v>
       </c>
-      <c r="Y22" s="73" t="s">
+      <c r="Y22" s="69" t="s">
         <v>240</v>
       </c>
-      <c r="Z22" s="73"/>
-      <c r="AA22" s="73"/>
-      <c r="AB22" s="73"/>
+      <c r="Z22" s="69"/>
+      <c r="AA22" s="69"/>
+      <c r="AB22" s="69"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
@@ -10033,16 +10066,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:AS2"/>
+    <mergeCell ref="Y18:AS18"/>
+    <mergeCell ref="Y13:AA13"/>
+    <mergeCell ref="Y14:AA14"/>
+    <mergeCell ref="Y15:AA15"/>
     <mergeCell ref="Y22:AB22"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="N3:S3"/>
     <mergeCell ref="O18:W18"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:AS2"/>
-    <mergeCell ref="Y18:AS18"/>
-    <mergeCell ref="Y13:AA13"/>
-    <mergeCell ref="Y14:AA14"/>
-    <mergeCell ref="Y15:AA15"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10076,7 +10109,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{877C88B0-3D7B-4586-98D6-71E94B4FEF77}">
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -10247,22 +10280,22 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>93</v>
       </c>
@@ -10270,22 +10303,22 @@
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I38" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I39" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G40" t="s">
         <v>257</v>
       </c>
@@ -10293,7 +10326,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G41" t="s">
         <v>258</v>
       </c>
@@ -10301,22 +10334,22 @@
         <v>250</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I42" s="60" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I43" s="60" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I44" s="59" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>94</v>
       </c>
@@ -10327,22 +10360,25 @@
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I46" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I47" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="I48" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J48" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G49" t="s">
         <v>247</v>
       </c>
@@ -10353,7 +10389,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G50" t="s">
         <v>248</v>
       </c>
@@ -10364,7 +10400,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
       <c r="G51" t="s">
         <v>255</v>
       </c>
@@ -10375,223 +10411,291 @@
         <v>253</v>
       </c>
     </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
       <c r="I52" s="59" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
       <c r="I53" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>96</v>
       </c>
       <c r="E55" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" t="s">
+      <c r="G55" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I56" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="J56" s="74" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I57" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="J57" s="74" t="s">
+        <v>266</v>
+      </c>
+      <c r="K57" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I58" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="J58" s="74" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I59" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="J59" s="75" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I60" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="J60" s="75" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I61" s="74" t="s">
+        <v>246</v>
+      </c>
+      <c r="J61" s="74"/>
+    </row>
+    <row r="62" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I62" s="74" t="s">
+        <v>251</v>
+      </c>
+      <c r="J62" s="74"/>
+    </row>
+    <row r="63" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I63" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="J63" s="75" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="64" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
         <v>97</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E64" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" t="s">
+      <c r="I64" s="74"/>
+      <c r="J64" s="74"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
         <v>98</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E65" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" t="s">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" t="s">
-        <v>101</v>
-      </c>
-      <c r="E60" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B65" s="58" t="s">
-        <v>128</v>
-      </c>
-      <c r="D65" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B66" s="60" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B67" s="59" t="s">
-        <v>130</v>
-      </c>
-      <c r="D67" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E68" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B69" s="58" t="s">
-        <v>104</v>
-      </c>
-      <c r="D69" t="s">
-        <v>261</v>
-      </c>
-      <c r="E69" t="s">
-        <v>263</v>
+      <c r="B69" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B70" s="60" t="s">
-        <v>105</v>
-      </c>
-      <c r="E70" t="s">
-        <v>264</v>
+      <c r="B70" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B71" s="59" t="s">
-        <v>106</v>
-      </c>
-      <c r="D71" t="s">
-        <v>262</v>
-      </c>
-      <c r="E71" t="s">
-        <v>141</v>
+      <c r="B71" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
-        <v>107</v>
-      </c>
-      <c r="E72" t="s">
-        <v>265</v>
+        <v>127</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B73" t="s">
-        <v>108</v>
+      <c r="B73" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="D73" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B74" t="s">
-        <v>109</v>
+      <c r="B74" s="60" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B75" t="s">
-        <v>110</v>
+      <c r="B75" s="59" t="s">
+        <v>130</v>
+      </c>
+      <c r="D75" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="E76" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B77" t="s">
-        <v>112</v>
+      <c r="B77" s="58" t="s">
+        <v>104</v>
+      </c>
+      <c r="D77" t="s">
+        <v>261</v>
       </c>
       <c r="E77" t="s">
-        <v>142</v>
+        <v>263</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B78" t="s">
-        <v>131</v>
+      <c r="B78" s="60" t="s">
+        <v>105</v>
       </c>
       <c r="E78" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B79" t="s">
-        <v>132</v>
+      <c r="B79" s="59" t="s">
+        <v>106</v>
+      </c>
+      <c r="D79" t="s">
+        <v>262</v>
       </c>
       <c r="E79" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="E80" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>134</v>
-      </c>
-      <c r="E81" t="s">
-        <v>142</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>135</v>
+        <v>109</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>111</v>
+      </c>
+      <c r="E84" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>112</v>
+      </c>
+      <c r="E85" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>131</v>
+      </c>
+      <c r="E86" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>132</v>
+      </c>
+      <c r="E87" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>133</v>
+      </c>
+      <c r="E88" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>134</v>
+      </c>
+      <c r="E89" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
         <v>136</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C91" t="s">
         <v>137</v>
       </c>
     </row>
@@ -10599,4 +10703,48 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC00DF4-147D-4096-AA5C-2C8738D449D0}">
+  <dimension ref="B3:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>272</v>
+      </c>
+      <c r="E3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated disassembly some more Moved PM2528 footprints/3D to subfolder
</commit_message>
<xml_diff>
--- a/Data/Info.xlsx
+++ b/Data/Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77490ADA-51A1-4349-9C52-8A9C9B4381CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7F18AE-599E-4B4C-8B65-3AC38681C0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="282">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -873,6 +873,24 @@
   </si>
   <si>
     <t>D6</t>
+  </si>
+  <si>
+    <t>Will be written out to Extmem</t>
+  </si>
+  <si>
+    <t>Assembly</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>Set  = CFI active</t>
+  </si>
+  <si>
+    <t>F0</t>
+  </si>
+  <si>
+    <t>Set = Overload active</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1377,9 +1395,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1392,8 +1407,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8672,29 +8688,29 @@
       <c r="AS2" s="64"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>241</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="K3" s="70" t="s">
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="K3" s="69" t="s">
         <v>171</v>
       </c>
-      <c r="L3" s="70"/>
+      <c r="L3" s="69"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="70" t="s">
+      <c r="N3" s="69" t="s">
         <v>172</v>
       </c>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="70"/>
-      <c r="S3" s="70"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="69"/>
+      <c r="R3" s="69"/>
+      <c r="S3" s="69"/>
     </row>
     <row r="4" spans="2:45" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -9170,11 +9186,11 @@
       <c r="S13" s="56">
         <v>0</v>
       </c>
-      <c r="Y13" s="71" t="s">
+      <c r="Y13" s="70" t="s">
         <v>215</v>
       </c>
-      <c r="Z13" s="71"/>
-      <c r="AA13" s="71"/>
+      <c r="Z13" s="70"/>
+      <c r="AA13" s="70"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9183,11 +9199,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="Y14" s="72" t="s">
+      <c r="Y14" s="71" t="s">
         <v>234</v>
       </c>
-      <c r="Z14" s="72"/>
-      <c r="AA14" s="72"/>
+      <c r="Z14" s="71"/>
+      <c r="AA14" s="71"/>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9198,11 +9214,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="Y15" s="73" t="s">
+      <c r="Y15" s="72" t="s">
         <v>235</v>
       </c>
-      <c r="Z15" s="73"/>
-      <c r="AA15" s="73"/>
+      <c r="Z15" s="72"/>
+      <c r="AA15" s="72"/>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9213,40 +9229,40 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="15:45" x14ac:dyDescent="0.25">
-      <c r="O18" s="70" t="s">
+      <c r="O18" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
-      <c r="V18" s="70"/>
-      <c r="W18" s="70"/>
-      <c r="Y18" s="70" t="s">
+      <c r="P18" s="69"/>
+      <c r="Q18" s="69"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="69"/>
+      <c r="U18" s="69"/>
+      <c r="V18" s="69"/>
+      <c r="W18" s="69"/>
+      <c r="Y18" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="Z18" s="70"/>
-      <c r="AA18" s="70"/>
-      <c r="AB18" s="70"/>
-      <c r="AC18" s="70"/>
-      <c r="AD18" s="70"/>
-      <c r="AE18" s="70"/>
-      <c r="AF18" s="70"/>
-      <c r="AG18" s="70"/>
-      <c r="AH18" s="70"/>
-      <c r="AI18" s="70"/>
-      <c r="AJ18" s="70"/>
-      <c r="AK18" s="70"/>
-      <c r="AL18" s="70"/>
-      <c r="AM18" s="70"/>
-      <c r="AN18" s="70"/>
-      <c r="AO18" s="70"/>
-      <c r="AP18" s="70"/>
-      <c r="AQ18" s="70"/>
-      <c r="AR18" s="70"/>
-      <c r="AS18" s="70"/>
+      <c r="Z18" s="69"/>
+      <c r="AA18" s="69"/>
+      <c r="AB18" s="69"/>
+      <c r="AC18" s="69"/>
+      <c r="AD18" s="69"/>
+      <c r="AE18" s="69"/>
+      <c r="AF18" s="69"/>
+      <c r="AG18" s="69"/>
+      <c r="AH18" s="69"/>
+      <c r="AI18" s="69"/>
+      <c r="AJ18" s="69"/>
+      <c r="AK18" s="69"/>
+      <c r="AL18" s="69"/>
+      <c r="AM18" s="69"/>
+      <c r="AN18" s="69"/>
+      <c r="AO18" s="69"/>
+      <c r="AP18" s="69"/>
+      <c r="AQ18" s="69"/>
+      <c r="AR18" s="69"/>
+      <c r="AS18" s="69"/>
     </row>
     <row r="19" spans="15:45" x14ac:dyDescent="0.25">
       <c r="P19" s="46" t="s">
@@ -9416,12 +9432,12 @@
       <c r="U22" s="48" t="s">
         <v>212</v>
       </c>
-      <c r="Y22" s="69" t="s">
+      <c r="Y22" s="73" t="s">
         <v>240</v>
       </c>
-      <c r="Z22" s="69"/>
-      <c r="AA22" s="69"/>
-      <c r="AB22" s="69"/>
+      <c r="Z22" s="73"/>
+      <c r="AA22" s="73"/>
+      <c r="AB22" s="73"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
@@ -10066,16 +10082,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="Y22:AB22"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="O18:W18"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="B2:AS2"/>
     <mergeCell ref="Y18:AS18"/>
     <mergeCell ref="Y13:AA13"/>
     <mergeCell ref="Y14:AA14"/>
     <mergeCell ref="Y15:AA15"/>
-    <mergeCell ref="Y22:AB22"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="O18:W18"/>
-    <mergeCell ref="B3:I3"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10089,7 +10105,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C115D6F0-6F20-429E-A21E-CAF81A83ED63}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -10100,6 +10116,27 @@
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B7" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>278</v>
+      </c>
+      <c r="B8" t="s">
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -10441,7 +10478,7 @@
       <c r="I56" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="J56" s="74" t="s">
+      <c r="J56" t="s">
         <v>266</v>
       </c>
     </row>
@@ -10449,7 +10486,7 @@
       <c r="I57" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="J57" s="74" t="s">
+      <c r="J57" t="s">
         <v>266</v>
       </c>
       <c r="K57" t="s">
@@ -10460,7 +10497,7 @@
       <c r="I58" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="J58" s="74" t="s">
+      <c r="J58" t="s">
         <v>266</v>
       </c>
     </row>
@@ -10468,7 +10505,7 @@
       <c r="I59" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="J59" s="75" t="s">
+      <c r="J59" t="s">
         <v>266</v>
       </c>
     </row>
@@ -10476,27 +10513,25 @@
       <c r="I60" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="J60" s="75" t="s">
+      <c r="J60" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I61" s="74" t="s">
+      <c r="I61" t="s">
         <v>246</v>
       </c>
-      <c r="J61" s="74"/>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I62" s="74" t="s">
+      <c r="I62" t="s">
         <v>251</v>
       </c>
-      <c r="J62" s="74"/>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
       <c r="I63" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="J63" s="75" t="s">
+      <c r="J63" t="s">
         <v>266</v>
       </c>
     </row>
@@ -10507,8 +10542,6 @@
       <c r="E64" t="s">
         <v>142</v>
       </c>
-      <c r="I64" s="74"/>
-      <c r="J64" s="74"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
@@ -10623,22 +10656,25 @@
         <v>265</v>
       </c>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="K83" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>111</v>
       </c>
@@ -10646,7 +10682,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>112</v>
       </c>
@@ -10654,7 +10690,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>131</v>
       </c>
@@ -10662,7 +10698,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>132</v>
       </c>
@@ -10670,7 +10706,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>133</v>
       </c>
@@ -10678,7 +10714,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>134</v>
       </c>
@@ -10686,12 +10722,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>136</v>
       </c>

</xml_diff>

<commit_message>
More disassembly More info in Info-Excel-sheet
</commit_message>
<xml_diff>
--- a/Data/Info.xlsx
+++ b/Data/Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7F18AE-599E-4B4C-8B65-3AC38681C0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BF2B8C-3A11-44A6-9B7E-891E5ECEC582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="256">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -266,66 +266,6 @@
     <t>Internal Memory</t>
   </si>
   <si>
-    <t>INTMEM_00</t>
-  </si>
-  <si>
-    <t>INTMEM_01</t>
-  </si>
-  <si>
-    <t>INTMEM_02</t>
-  </si>
-  <si>
-    <t>INTMEM_03</t>
-  </si>
-  <si>
-    <t>INTMEM_04</t>
-  </si>
-  <si>
-    <t>INTMEM_05</t>
-  </si>
-  <si>
-    <t>INTMEM_06</t>
-  </si>
-  <si>
-    <t>INTMEM_07</t>
-  </si>
-  <si>
-    <t>INTMEM_08</t>
-  </si>
-  <si>
-    <t>INTMEM_09</t>
-  </si>
-  <si>
-    <t>INTMEM_10</t>
-  </si>
-  <si>
-    <t>INTMEM_11</t>
-  </si>
-  <si>
-    <t>INTMEM_12</t>
-  </si>
-  <si>
-    <t>INTMEM_13</t>
-  </si>
-  <si>
-    <t>INTMEM_14</t>
-  </si>
-  <si>
-    <t>INTMEM_15</t>
-  </si>
-  <si>
-    <t>INTMEM_16</t>
-  </si>
-  <si>
-    <t>INTMEM_17</t>
-  </si>
-  <si>
-    <t>INTMEM_18</t>
-  </si>
-  <si>
-    <t>INTMEM_19</t>
-  </si>
-  <si>
     <t>INTMEM_20</t>
   </si>
   <si>
@@ -386,42 +326,6 @@
     <t>INTMEM_39</t>
   </si>
   <si>
-    <t>INTMEM_0A</t>
-  </si>
-  <si>
-    <t>INTMEM_0B</t>
-  </si>
-  <si>
-    <t>INTMEM_0C</t>
-  </si>
-  <si>
-    <t>INTMEM_0D</t>
-  </si>
-  <si>
-    <t>INTMEM_0E</t>
-  </si>
-  <si>
-    <t>INTMEM_0F</t>
-  </si>
-  <si>
-    <t>INTMEM_1A</t>
-  </si>
-  <si>
-    <t>INTMEM_1B</t>
-  </si>
-  <si>
-    <t>INTMEM_1C</t>
-  </si>
-  <si>
-    <t>INTMEM_1D</t>
-  </si>
-  <si>
-    <t>INTMEM_1E</t>
-  </si>
-  <si>
-    <t>INTMEM_1F</t>
-  </si>
-  <si>
     <t>INTMEM_2A</t>
   </si>
   <si>
@@ -728,9 +632,6 @@
     <t>(illegal)</t>
   </si>
   <si>
-    <t>(Low = on)</t>
-  </si>
-  <si>
     <t>+</t>
   </si>
   <si>
@@ -740,9 +641,6 @@
     <t>REM</t>
   </si>
   <si>
-    <t>(low=on)</t>
-  </si>
-  <si>
     <t>Ω2W</t>
   </si>
   <si>
@@ -818,12 +716,6 @@
     <t>1=on</t>
   </si>
   <si>
-    <t>Autoranging?</t>
-  </si>
-  <si>
-    <t>Bitpattern for Function-indicators?</t>
-  </si>
-  <si>
     <t>0x01</t>
   </si>
   <si>
@@ -845,9 +737,6 @@
     <t>0xf0</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>something with Galvanic Isolation Card</t>
   </si>
   <si>
@@ -891,6 +780,39 @@
   </si>
   <si>
     <t>Set = Overload active</t>
+  </si>
+  <si>
+    <t>Read by TMRIRQ</t>
+  </si>
+  <si>
+    <t>Hardware</t>
+  </si>
+  <si>
+    <t>P1 = INT0 | ENI | WDOG | POL | HSM | SRUP | SAZ | AZ</t>
+  </si>
+  <si>
+    <t>f;</t>
+  </si>
+  <si>
+    <t>TriggerMode</t>
+  </si>
+  <si>
+    <t>Autoranging</t>
+  </si>
+  <si>
+    <t>Bitpattern for Function-indicators</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>0000=VDC, 0001=VAC, 0010=VDCAC, 0011=O2W</t>
+  </si>
+  <si>
+    <t>00100=O4W, 00101ADC, 0110=ADCAC, 0111=C</t>
+  </si>
+  <si>
+    <t>1000=Vhf, 1001=Vpeak</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1395,6 +1317,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1407,14 +1332,82 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -7067,7 +7060,7 @@
     </row>
     <row r="2" spans="1:29" ht="24" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D2" s="64" t="s">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="E2" s="64"/>
       <c r="F2" s="64"/>
@@ -7097,7 +7090,7 @@
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="D3" s="65" t="s">
-        <v>170</v>
+        <v>138</v>
       </c>
       <c r="E3" s="62"/>
       <c r="F3" s="62"/>
@@ -7107,14 +7100,14 @@
       <c r="J3" s="62"/>
       <c r="K3" s="63"/>
       <c r="N3" s="66" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="O3" s="67"/>
       <c r="P3" s="67"/>
       <c r="Q3" s="67"/>
       <c r="R3" s="18"/>
       <c r="S3" s="67" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="T3" s="67"/>
       <c r="U3" s="67"/>
@@ -7144,16 +7137,16 @@
         <v>58</v>
       </c>
       <c r="H4" s="43" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="I4" s="43" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="J4" s="43" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="K4" s="23" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="N4" s="19" t="s">
         <v>51</v>
@@ -7190,10 +7183,10 @@
         <v>64</v>
       </c>
       <c r="AB4" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC4" s="26" t="s">
         <v>61</v>
-      </c>
-      <c r="AC4" s="26" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
@@ -7230,7 +7223,7 @@
         <v>63</v>
       </c>
       <c r="L6" s="32" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="N6" s="31">
         <v>1</v>
@@ -7303,7 +7296,7 @@
         <v>63</v>
       </c>
       <c r="L7" s="32" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="N7" s="31">
         <v>1</v>
@@ -7376,7 +7369,7 @@
         <v>63</v>
       </c>
       <c r="L8" s="32" t="s">
-        <v>152</v>
+        <v>120</v>
       </c>
       <c r="N8" s="31">
         <v>1</v>
@@ -7449,7 +7442,7 @@
         <v>63</v>
       </c>
       <c r="L9" s="32" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="N9" s="31">
         <v>1</v>
@@ -7523,7 +7516,7 @@
         <v>63</v>
       </c>
       <c r="L10" s="32" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="N10" s="31">
         <v>1</v>
@@ -7563,12 +7556,10 @@
       </c>
       <c r="AA10" s="32"/>
       <c r="AB10" s="32">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC10" s="35">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
@@ -7597,7 +7588,7 @@
         <v>63</v>
       </c>
       <c r="L11" s="32" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="N11" s="31">
         <v>1</v>
@@ -7637,12 +7628,10 @@
       </c>
       <c r="AA11" s="32"/>
       <c r="AB11" s="32">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC11" s="35">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.25">
@@ -7671,7 +7660,7 @@
         <v>63</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="N12" s="31">
         <v>1</v>
@@ -7711,12 +7700,10 @@
       </c>
       <c r="AA12" s="32"/>
       <c r="AB12" s="32">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC12" s="35">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
@@ -7745,7 +7732,7 @@
         <v>63</v>
       </c>
       <c r="L13" s="32" t="s">
-        <v>157</v>
+        <v>125</v>
       </c>
       <c r="N13" s="31">
         <v>1</v>
@@ -7785,12 +7772,10 @@
       </c>
       <c r="AA13" s="32"/>
       <c r="AB13" s="32">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC13" s="35">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
@@ -7819,7 +7804,7 @@
         <v>63</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="N14" s="31">
         <v>1</v>
@@ -7859,12 +7844,10 @@
       </c>
       <c r="AA14" s="32"/>
       <c r="AB14" s="32">
-        <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="35">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
@@ -7893,7 +7876,7 @@
         <v>63</v>
       </c>
       <c r="L15" s="32" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="N15" s="31">
         <v>1</v>
@@ -7933,12 +7916,10 @@
       </c>
       <c r="AA15" s="32"/>
       <c r="AB15" s="32">
-        <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC15" s="35">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
@@ -7967,7 +7948,7 @@
         <v>63</v>
       </c>
       <c r="L16" s="32" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="N16" s="31">
         <v>1</v>
@@ -8007,12 +7988,10 @@
       </c>
       <c r="AA16" s="32"/>
       <c r="AB16" s="32">
-        <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC16" s="35">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="4:33" x14ac:dyDescent="0.25">
@@ -8041,7 +8020,7 @@
         <v>63</v>
       </c>
       <c r="L17" s="32" t="s">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="N17" s="31">
         <v>1</v>
@@ -8081,12 +8060,10 @@
       </c>
       <c r="AA17" s="32"/>
       <c r="AB17" s="32">
-        <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC17" s="35">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="4:33" x14ac:dyDescent="0.25">
@@ -8115,7 +8092,7 @@
         <v>63</v>
       </c>
       <c r="L18" s="32" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="N18" s="31">
         <v>0</v>
@@ -8190,7 +8167,7 @@
         <v>63</v>
       </c>
       <c r="L19" s="32" t="s">
-        <v>163</v>
+        <v>131</v>
       </c>
       <c r="N19" s="31">
         <v>0</v>
@@ -8264,7 +8241,7 @@
         <v>63</v>
       </c>
       <c r="L20" s="32" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="N20" s="31">
         <v>0</v>
@@ -8338,7 +8315,7 @@
         <v>63</v>
       </c>
       <c r="L21" s="32" t="s">
-        <v>165</v>
+        <v>133</v>
       </c>
       <c r="N21" s="36">
         <v>0</v>
@@ -8603,7 +8580,7 @@
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="X6:Z21 AB6:AC21">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8688,29 +8665,29 @@
       <c r="AS2" s="64"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B3" s="69" t="s">
-        <v>241</v>
-      </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="K3" s="69" t="s">
-        <v>171</v>
-      </c>
-      <c r="L3" s="69"/>
+      <c r="B3" s="70" t="s">
+        <v>207</v>
+      </c>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="K3" s="70" t="s">
+        <v>139</v>
+      </c>
+      <c r="L3" s="70"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="69" t="s">
-        <v>172</v>
-      </c>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
+      <c r="N3" s="70" t="s">
+        <v>140</v>
+      </c>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="70"/>
+      <c r="S3" s="70"/>
     </row>
     <row r="4" spans="2:45" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -8726,61 +8703,61 @@
         <v>58</v>
       </c>
       <c r="F4" s="43" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="G4" s="43" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="H4" s="43" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="I4" s="43" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="K4" s="46" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="L4" s="46" t="s">
-        <v>167</v>
+        <v>135</v>
       </c>
       <c r="M4" s="42"/>
       <c r="N4" s="46" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="P4" s="46" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="Q4" s="46" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="R4" s="46" t="s">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="S4" s="46" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N5" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="O5" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="P5" t="s">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="Q5" t="s">
-        <v>175</v>
+        <v>143</v>
       </c>
       <c r="R5" t="s">
-        <v>176</v>
+        <v>144</v>
       </c>
       <c r="S5" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="U5" s="32"/>
       <c r="V5" s="32"/>
@@ -8862,8 +8839,8 @@
       <c r="I7" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="K7" s="32">
-        <v>0</v>
+      <c r="K7" s="32" t="s">
+        <v>252</v>
       </c>
       <c r="L7" s="32">
         <v>1</v>
@@ -9186,11 +9163,11 @@
       <c r="S13" s="56">
         <v>0</v>
       </c>
-      <c r="Y13" s="70" t="s">
-        <v>215</v>
-      </c>
-      <c r="Z13" s="70"/>
-      <c r="AA13" s="70"/>
+      <c r="Y13" s="71" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z13" s="71"/>
+      <c r="AA13" s="71"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9199,26 +9176,26 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="Y14" s="71" t="s">
-        <v>234</v>
-      </c>
-      <c r="Z14" s="71"/>
-      <c r="AA14" s="71"/>
+      <c r="Y14" s="72" t="s">
+        <v>200</v>
+      </c>
+      <c r="Z14" s="72"/>
+      <c r="AA14" s="72"/>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
-        <v>242</v>
+        <v>208</v>
       </c>
       <c r="O15" s="32"/>
       <c r="P15" s="32"/>
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="Y15" s="72" t="s">
-        <v>235</v>
-      </c>
-      <c r="Z15" s="72"/>
-      <c r="AA15" s="72"/>
+      <c r="Y15" s="73" t="s">
+        <v>201</v>
+      </c>
+      <c r="Z15" s="73"/>
+      <c r="AA15" s="73"/>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9229,159 +9206,153 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="15:45" x14ac:dyDescent="0.25">
-      <c r="O18" s="69" t="s">
-        <v>166</v>
-      </c>
-      <c r="P18" s="69"/>
-      <c r="Q18" s="69"/>
-      <c r="R18" s="69"/>
-      <c r="S18" s="69"/>
-      <c r="T18" s="69"/>
-      <c r="U18" s="69"/>
-      <c r="V18" s="69"/>
-      <c r="W18" s="69"/>
-      <c r="Y18" s="69" t="s">
-        <v>216</v>
-      </c>
-      <c r="Z18" s="69"/>
-      <c r="AA18" s="69"/>
-      <c r="AB18" s="69"/>
-      <c r="AC18" s="69"/>
-      <c r="AD18" s="69"/>
-      <c r="AE18" s="69"/>
-      <c r="AF18" s="69"/>
-      <c r="AG18" s="69"/>
-      <c r="AH18" s="69"/>
-      <c r="AI18" s="69"/>
-      <c r="AJ18" s="69"/>
-      <c r="AK18" s="69"/>
-      <c r="AL18" s="69"/>
-      <c r="AM18" s="69"/>
-      <c r="AN18" s="69"/>
-      <c r="AO18" s="69"/>
-      <c r="AP18" s="69"/>
-      <c r="AQ18" s="69"/>
-      <c r="AR18" s="69"/>
-      <c r="AS18" s="69"/>
+      <c r="O18" s="70" t="s">
+        <v>134</v>
+      </c>
+      <c r="P18" s="70"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="70"/>
+      <c r="S18" s="70"/>
+      <c r="T18" s="70"/>
+      <c r="U18" s="70"/>
+      <c r="V18" s="70"/>
+      <c r="W18" s="70"/>
+      <c r="Y18" s="70" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z18" s="70"/>
+      <c r="AA18" s="70"/>
+      <c r="AB18" s="70"/>
+      <c r="AC18" s="70"/>
+      <c r="AD18" s="70"/>
+      <c r="AE18" s="70"/>
+      <c r="AF18" s="70"/>
+      <c r="AG18" s="70"/>
+      <c r="AH18" s="70"/>
+      <c r="AI18" s="70"/>
+      <c r="AJ18" s="70"/>
+      <c r="AK18" s="70"/>
+      <c r="AL18" s="70"/>
+      <c r="AM18" s="70"/>
+      <c r="AN18" s="70"/>
+      <c r="AO18" s="70"/>
+      <c r="AP18" s="70"/>
+      <c r="AQ18" s="70"/>
+      <c r="AR18" s="70"/>
+      <c r="AS18" s="70"/>
     </row>
     <row r="19" spans="15:45" x14ac:dyDescent="0.25">
       <c r="P19" s="46" t="s">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="Q19" s="46" t="s">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="R19" s="46" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="S19" s="46" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
       <c r="T19" s="46"/>
       <c r="U19" s="46" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
       <c r="V19" s="57"/>
       <c r="W19" s="46" t="s">
-        <v>214</v>
+        <v>182</v>
       </c>
       <c r="Y19" s="46" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="Z19" s="46" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="AA19" s="46" t="s">
-        <v>188</v>
+        <v>156</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>189</v>
+        <v>157</v>
       </c>
       <c r="AD19" s="46" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
       <c r="AE19" s="46" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="AF19" s="46" t="s">
-        <v>209</v>
+        <v>177</v>
       </c>
       <c r="AG19" s="46" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
       <c r="AI19" s="51" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="AJ19" s="51" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="AK19" s="51" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="AL19" s="51" t="s">
-        <v>196</v>
-      </c>
-      <c r="AM19" t="s">
-        <v>231</v>
+        <v>164</v>
       </c>
       <c r="AO19" s="46" t="s">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="AP19" s="46" t="s">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="AQ19" s="46" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="AR19" s="46" t="s">
-        <v>185</v>
-      </c>
-      <c r="AS19" t="s">
-        <v>227</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O21" s="46" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="P21" s="48" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
       <c r="Q21" s="48"/>
       <c r="R21" s="48" t="s">
-        <v>217</v>
+        <v>185</v>
       </c>
       <c r="S21" s="48" t="s">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="T21" s="48"/>
       <c r="U21" s="48" t="s">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="Y21" s="56" t="s">
-        <v>239</v>
+        <v>205</v>
       </c>
       <c r="Z21" s="56" t="s">
-        <v>238</v>
+        <v>204</v>
       </c>
       <c r="AA21" s="56" t="s">
-        <v>237</v>
+        <v>203</v>
       </c>
       <c r="AB21" s="56" t="s">
-        <v>236</v>
+        <v>202</v>
       </c>
       <c r="AC21" s="32"/>
       <c r="AD21" s="53" t="s">
-        <v>222</v>
+        <v>190</v>
       </c>
       <c r="AE21" s="53" t="s">
         <v>10</v>
       </c>
       <c r="AF21" s="53" t="s">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="AG21" s="53" t="s">
-        <v>228</v>
+        <v>195</v>
       </c>
       <c r="AI21" s="32">
         <v>0</v>
@@ -9396,7 +9367,7 @@
         <v>0</v>
       </c>
       <c r="AM21" s="52" t="s">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="AO21" s="32">
         <v>0</v>
@@ -9411,33 +9382,33 @@
         <v>0</v>
       </c>
       <c r="AS21" s="55" t="s">
-        <v>218</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O22" s="46" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="P22" s="48" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
       <c r="Q22" s="48"/>
       <c r="R22" s="48" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="S22" s="48" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
       <c r="T22" s="48"/>
       <c r="U22" s="48" t="s">
-        <v>212</v>
-      </c>
-      <c r="Y22" s="73" t="s">
-        <v>240</v>
-      </c>
-      <c r="Z22" s="73"/>
-      <c r="AA22" s="73"/>
-      <c r="AB22" s="73"/>
+        <v>180</v>
+      </c>
+      <c r="Y22" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="Z22" s="69"/>
+      <c r="AA22" s="69"/>
+      <c r="AB22" s="69"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
@@ -9456,7 +9427,7 @@
         <v>1</v>
       </c>
       <c r="AM22" s="52" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="AO22" s="32">
         <v>0</v>
@@ -9471,28 +9442,28 @@
         <v>1</v>
       </c>
       <c r="AS22" s="55" t="s">
-        <v>219</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O23" s="46" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="P23" s="48" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="Q23" s="48" t="s">
         <v>67</v>
       </c>
       <c r="R23" s="48" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="S23" s="48" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="T23" s="48"/>
       <c r="U23" s="48" t="s">
-        <v>211</v>
+        <v>179</v>
       </c>
       <c r="AC23" s="32"/>
       <c r="AD23" s="32"/>
@@ -9512,7 +9483,7 @@
         <v>0</v>
       </c>
       <c r="AM23" s="52" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
       <c r="AO23" s="32">
         <v>0</v>
@@ -9527,28 +9498,28 @@
         <v>0</v>
       </c>
       <c r="AS23" s="55" t="s">
-        <v>220</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O24" s="46" t="s">
-        <v>196</v>
+        <v>164</v>
       </c>
       <c r="P24" s="48" t="s">
-        <v>202</v>
+        <v>170</v>
       </c>
       <c r="Q24" s="48" t="s">
         <v>43</v>
       </c>
       <c r="R24" s="48" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="S24" s="48" t="s">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="T24" s="48"/>
       <c r="U24" s="48" t="s">
-        <v>210</v>
+        <v>178</v>
       </c>
       <c r="AC24" s="32"/>
       <c r="AD24" s="32"/>
@@ -9568,7 +9539,7 @@
         <v>1</v>
       </c>
       <c r="AM24" s="52" t="s">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="AO24" s="32">
         <v>0</v>
@@ -9583,7 +9554,7 @@
         <v>1</v>
       </c>
       <c r="AS24" s="55" t="s">
-        <v>217</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="15:45" x14ac:dyDescent="0.25">
@@ -9605,7 +9576,7 @@
         <v>0</v>
       </c>
       <c r="AM25" s="52" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="AO25" s="32">
         <v>0</v>
@@ -9620,15 +9591,15 @@
         <v>0</v>
       </c>
       <c r="AS25" s="55" t="s">
-        <v>221</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O26" s="46" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
       <c r="W26" s="49" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
       <c r="AC26" s="32"/>
       <c r="AD26" s="32"/>
@@ -9648,7 +9619,7 @@
         <v>1</v>
       </c>
       <c r="AM26" s="52" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="AO26" s="32">
         <v>0</v>
@@ -9663,15 +9634,15 @@
         <v>1</v>
       </c>
       <c r="AS26" s="55" t="s">
-        <v>221</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O27" s="46" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="W27" s="52" t="s">
-        <v>230</v>
+        <v>197</v>
       </c>
       <c r="AC27" s="32"/>
       <c r="AD27" s="32"/>
@@ -9691,7 +9662,7 @@
         <v>0</v>
       </c>
       <c r="AM27" s="52" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="AO27" s="32">
         <v>0</v>
@@ -9706,15 +9677,15 @@
         <v>0</v>
       </c>
       <c r="AS27" s="55" t="s">
-        <v>223</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O28" s="46" t="s">
-        <v>209</v>
+        <v>177</v>
       </c>
       <c r="W28" s="49" t="s">
-        <v>210</v>
+        <v>178</v>
       </c>
       <c r="AC28" s="32"/>
       <c r="AD28" s="50"/>
@@ -9734,7 +9705,7 @@
         <v>1</v>
       </c>
       <c r="AM28" s="52" t="s">
-        <v>217</v>
+        <v>185</v>
       </c>
       <c r="AO28" s="50">
         <v>0</v>
@@ -9749,12 +9720,12 @@
         <v>1</v>
       </c>
       <c r="AS28" t="s">
-        <v>225</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O29" s="54" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
       <c r="AC29" s="32"/>
       <c r="AD29" s="32"/>
@@ -9789,7 +9760,7 @@
         <v>0</v>
       </c>
       <c r="AS29" s="55" t="s">
-        <v>224</v>
+        <v>192</v>
       </c>
     </row>
     <row r="30" spans="15:45" x14ac:dyDescent="0.25">
@@ -9831,10 +9802,10 @@
     </row>
     <row r="31" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O31" s="46" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="W31" s="49" t="s">
-        <v>204</v>
+        <v>181</v>
       </c>
       <c r="AC31" s="32"/>
       <c r="AD31" s="50"/>
@@ -9854,7 +9825,7 @@
         <v>0</v>
       </c>
       <c r="AM31" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO31" s="50">
         <v>1</v>
@@ -9869,15 +9840,15 @@
         <v>0</v>
       </c>
       <c r="AS31" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O32" s="46" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="W32" s="49" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="AD32" s="50"/>
       <c r="AE32" s="50"/>
@@ -9896,7 +9867,7 @@
         <v>1</v>
       </c>
       <c r="AM32" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO32" s="50">
         <v>1</v>
@@ -9911,15 +9882,15 @@
         <v>1</v>
       </c>
       <c r="AS32" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O33" s="46" t="s">
-        <v>188</v>
+        <v>156</v>
       </c>
       <c r="W33" s="49" t="s">
-        <v>202</v>
+        <v>171</v>
       </c>
       <c r="AD33" s="50"/>
       <c r="AE33" s="50"/>
@@ -9938,7 +9909,7 @@
         <v>0</v>
       </c>
       <c r="AM33" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO33" s="50">
         <v>1</v>
@@ -9953,15 +9924,15 @@
         <v>0</v>
       </c>
       <c r="AS33" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="15:45" x14ac:dyDescent="0.25">
       <c r="O34" s="46" t="s">
-        <v>189</v>
+        <v>157</v>
       </c>
       <c r="W34" s="49" t="s">
-        <v>213</v>
+        <v>172</v>
       </c>
       <c r="AD34" s="50"/>
       <c r="AE34" s="50"/>
@@ -9980,7 +9951,7 @@
         <v>1</v>
       </c>
       <c r="AM34" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO34" s="50">
         <v>1</v>
@@ -9995,7 +9966,7 @@
         <v>1</v>
       </c>
       <c r="AS34" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="15:45" x14ac:dyDescent="0.25">
@@ -10023,7 +9994,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO35" s="50">
         <v>1</v>
@@ -10038,7 +10009,7 @@
         <v>0</v>
       </c>
       <c r="AS35" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="15:45" x14ac:dyDescent="0.25">
@@ -10062,7 +10033,7 @@
         <v>1</v>
       </c>
       <c r="AM36" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
       <c r="AO36" s="50">
         <v>1</v>
@@ -10077,25 +10048,25 @@
         <v>1</v>
       </c>
       <c r="AS36" t="s">
-        <v>226</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:AS2"/>
+    <mergeCell ref="Y18:AS18"/>
+    <mergeCell ref="Y13:AA13"/>
+    <mergeCell ref="Y14:AA14"/>
+    <mergeCell ref="Y15:AA15"/>
     <mergeCell ref="Y22:AB22"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="N3:S3"/>
     <mergeCell ref="O18:W18"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:AS2"/>
-    <mergeCell ref="Y18:AS18"/>
-    <mergeCell ref="Y13:AA13"/>
-    <mergeCell ref="Y14:AA14"/>
-    <mergeCell ref="Y15:AA15"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10105,7 +10076,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C115D6F0-6F20-429E-A21E-CAF81A83ED63}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -10120,23 +10091,33 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>277</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>280</v>
+        <v>243</v>
       </c>
       <c r="B7" t="s">
-        <v>281</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>278</v>
+        <v>241</v>
       </c>
       <c r="B8" t="s">
-        <v>279</v>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -10146,7 +10127,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{877C88B0-3D7B-4586-98D6-71E94B4FEF77}">
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -10159,580 +10140,471 @@
     <col min="9" max="9" width="4.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="C4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E4" s="42" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>250</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="J8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>251</v>
+      </c>
+      <c r="I9" s="58" t="s">
+        <v>216</v>
+      </c>
+      <c r="J9" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I10" s="60" t="s">
+        <v>212</v>
+      </c>
+      <c r="J10" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I11" s="60" t="s">
+        <v>217</v>
+      </c>
+      <c r="J11" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I12" s="59" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="C13" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I14" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I16" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="J16" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>213</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="J17" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>214</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="J18" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>221</v>
+      </c>
+      <c r="I19" s="58" t="s">
+        <v>212</v>
+      </c>
+      <c r="J19" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I20" s="59" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="E23" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I24" s="9" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I25" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K25" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I26" s="9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I27" s="9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I28" s="9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I29" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I30" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I31" s="9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+      <c r="E32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I33" s="74" t="s">
+        <v>209</v>
+      </c>
+      <c r="J33" s="74"/>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I34" s="74" t="s">
+        <v>210</v>
+      </c>
+      <c r="J34" s="74"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I35" s="74" t="s">
+        <v>211</v>
+      </c>
+      <c r="J35" s="74"/>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I36" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="J36" s="74"/>
+    </row>
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I37" s="74" t="s">
+        <v>216</v>
+      </c>
+      <c r="J37" s="74"/>
+    </row>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I38" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="J38" s="74"/>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I39" s="74" t="s">
+        <v>217</v>
+      </c>
+      <c r="J39" s="74"/>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I40" s="74" t="s">
+        <v>218</v>
+      </c>
+      <c r="J40" s="74"/>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="E41" t="s">
+        <v>110</v>
+      </c>
+      <c r="G41" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="K43" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+      <c r="E44" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B49" s="58" t="s">
+        <v>96</v>
+      </c>
+      <c r="D49" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B50" s="60" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B51" s="59" t="s">
+        <v>98</v>
+      </c>
+      <c r="D51" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+      <c r="E52" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B53" s="58" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+      <c r="D53" t="s">
+        <v>225</v>
+      </c>
+      <c r="E53" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B54" s="60" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+      <c r="E54" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B55" s="59" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+      <c r="D55" t="s">
+        <v>226</v>
+      </c>
+      <c r="E55" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
+      <c r="E56" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
+    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
+    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
+      <c r="K59" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
+      <c r="E60" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>93</v>
-      </c>
-      <c r="E36" s="42" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I37" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I38" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I39" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="G40" t="s">
-        <v>257</v>
-      </c>
-      <c r="I40" s="9" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="G41" t="s">
-        <v>258</v>
-      </c>
-      <c r="I41" s="58" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I42" s="60" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I43" s="60" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I44" s="59" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
-        <v>94</v>
-      </c>
-      <c r="C45" t="s">
-        <v>254</v>
-      </c>
-      <c r="E45" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I46" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I47" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I48" t="s">
-        <v>245</v>
-      </c>
-      <c r="J48" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G49" t="s">
-        <v>247</v>
-      </c>
-      <c r="I49" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="J49" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G50" t="s">
-        <v>248</v>
-      </c>
-      <c r="I50" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="J50" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G51" t="s">
-        <v>255</v>
-      </c>
-      <c r="I51" s="58" t="s">
-        <v>246</v>
-      </c>
-      <c r="J51" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I52" s="59" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I53" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
-        <v>96</v>
-      </c>
-      <c r="E55" t="s">
-        <v>143</v>
-      </c>
-      <c r="G55" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I56" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="J56" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I57" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="J57" t="s">
-        <v>266</v>
-      </c>
-      <c r="K57" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I58" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="J58" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I59" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="J59" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I60" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="J60" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I61" t="s">
-        <v>246</v>
+      <c r="E61" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I62" t="s">
-        <v>251</v>
+      <c r="B62" t="s">
+        <v>99</v>
+      </c>
+      <c r="E62" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I63" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="J63" t="s">
-        <v>266</v>
+      <c r="B63" t="s">
+        <v>100</v>
+      </c>
+      <c r="E63" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E64" t="s">
-        <v>142</v>
+        <v>223</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E65" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B68" t="s">
-        <v>101</v>
-      </c>
-      <c r="E68" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B71" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B72" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B73" s="58" t="s">
-        <v>128</v>
-      </c>
-      <c r="D73" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B74" s="60" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B75" s="59" t="s">
-        <v>130</v>
-      </c>
-      <c r="D75" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B76" t="s">
-        <v>103</v>
-      </c>
-      <c r="E76" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B77" s="58" t="s">
         <v>104</v>
       </c>
-      <c r="D77" t="s">
-        <v>261</v>
-      </c>
-      <c r="E77" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B78" s="60" t="s">
+      <c r="C67" t="s">
         <v>105</v>
-      </c>
-      <c r="E78" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B79" s="59" t="s">
-        <v>106</v>
-      </c>
-      <c r="D79" t="s">
-        <v>262</v>
-      </c>
-      <c r="E79" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>107</v>
-      </c>
-      <c r="E80" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
-        <v>110</v>
-      </c>
-      <c r="K83" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>111</v>
-      </c>
-      <c r="E84" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B85" t="s">
-        <v>112</v>
-      </c>
-      <c r="E85" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B86" t="s">
-        <v>131</v>
-      </c>
-      <c r="E86" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B87" t="s">
-        <v>132</v>
-      </c>
-      <c r="E87" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
-        <v>133</v>
-      </c>
-      <c r="E88" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B89" t="s">
-        <v>134</v>
-      </c>
-      <c r="E89" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B90" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B91" t="s">
-        <v>136</v>
-      </c>
-      <c r="C91" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -10748,22 +10620,22 @@
   <sheetData>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>271</v>
+        <v>234</v>
       </c>
       <c r="C3" t="s">
-        <v>270</v>
+        <v>233</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>272</v>
+        <v>235</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>236</v>
       </c>
       <c r="F3" t="s">
-        <v>274</v>
+        <v>237</v>
       </c>
       <c r="G3" t="s">
-        <v>275</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Some more disassembly, optimize N20 schematics (naming of signals)
</commit_message>
<xml_diff>
--- a/Data/Info.xlsx
+++ b/Data/Info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CBC825-C00A-43B7-8180-C9D032046CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33D65CF-8F60-4EEE-8311-7836C4D235C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1686" uniqueCount="257">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -813,6 +813,9 @@
   </si>
   <si>
     <t>InstrumentMode_00</t>
+  </si>
+  <si>
+    <t>statusbyte? 0xF0 was HSM disabled, 0x00 was HSM enabled</t>
   </si>
 </sst>
 </file>
@@ -1317,9 +1320,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1331,6 +1331,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8594,29 +8597,29 @@
       <c r="AS2" s="64"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>204</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="K3" s="70" t="s">
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="K3" s="69" t="s">
         <v>136</v>
       </c>
-      <c r="L3" s="70"/>
+      <c r="L3" s="69"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="70" t="s">
+      <c r="N3" s="69" t="s">
         <v>137</v>
       </c>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="70"/>
-      <c r="S3" s="70"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="69"/>
+      <c r="R3" s="69"/>
+      <c r="S3" s="69"/>
     </row>
     <row r="4" spans="2:45" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -9092,11 +9095,11 @@
       <c r="S13" s="56">
         <v>0</v>
       </c>
-      <c r="Y13" s="71" t="s">
+      <c r="Y13" s="70" t="s">
         <v>180</v>
       </c>
-      <c r="Z13" s="71"/>
-      <c r="AA13" s="71"/>
+      <c r="Z13" s="70"/>
+      <c r="AA13" s="70"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9105,11 +9108,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="Y14" s="72" t="s">
+      <c r="Y14" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="Z14" s="72"/>
-      <c r="AA14" s="72"/>
+      <c r="Z14" s="71"/>
+      <c r="AA14" s="71"/>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9120,11 +9123,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="Y15" s="73" t="s">
+      <c r="Y15" s="72" t="s">
         <v>198</v>
       </c>
-      <c r="Z15" s="73"/>
-      <c r="AA15" s="73"/>
+      <c r="Z15" s="72"/>
+      <c r="AA15" s="72"/>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9135,40 +9138,40 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="15:45" x14ac:dyDescent="0.25">
-      <c r="O18" s="70" t="s">
+      <c r="O18" s="69" t="s">
         <v>131</v>
       </c>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
-      <c r="V18" s="70"/>
-      <c r="W18" s="70"/>
-      <c r="Y18" s="70" t="s">
+      <c r="P18" s="69"/>
+      <c r="Q18" s="69"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="69"/>
+      <c r="U18" s="69"/>
+      <c r="V18" s="69"/>
+      <c r="W18" s="69"/>
+      <c r="Y18" s="69" t="s">
         <v>181</v>
       </c>
-      <c r="Z18" s="70"/>
-      <c r="AA18" s="70"/>
-      <c r="AB18" s="70"/>
-      <c r="AC18" s="70"/>
-      <c r="AD18" s="70"/>
-      <c r="AE18" s="70"/>
-      <c r="AF18" s="70"/>
-      <c r="AG18" s="70"/>
-      <c r="AH18" s="70"/>
-      <c r="AI18" s="70"/>
-      <c r="AJ18" s="70"/>
-      <c r="AK18" s="70"/>
-      <c r="AL18" s="70"/>
-      <c r="AM18" s="70"/>
-      <c r="AN18" s="70"/>
-      <c r="AO18" s="70"/>
-      <c r="AP18" s="70"/>
-      <c r="AQ18" s="70"/>
-      <c r="AR18" s="70"/>
-      <c r="AS18" s="70"/>
+      <c r="Z18" s="69"/>
+      <c r="AA18" s="69"/>
+      <c r="AB18" s="69"/>
+      <c r="AC18" s="69"/>
+      <c r="AD18" s="69"/>
+      <c r="AE18" s="69"/>
+      <c r="AF18" s="69"/>
+      <c r="AG18" s="69"/>
+      <c r="AH18" s="69"/>
+      <c r="AI18" s="69"/>
+      <c r="AJ18" s="69"/>
+      <c r="AK18" s="69"/>
+      <c r="AL18" s="69"/>
+      <c r="AM18" s="69"/>
+      <c r="AN18" s="69"/>
+      <c r="AO18" s="69"/>
+      <c r="AP18" s="69"/>
+      <c r="AQ18" s="69"/>
+      <c r="AR18" s="69"/>
+      <c r="AS18" s="69"/>
     </row>
     <row r="19" spans="15:45" x14ac:dyDescent="0.25">
       <c r="P19" s="46" t="s">
@@ -9332,12 +9335,12 @@
       <c r="U22" s="48" t="s">
         <v>177</v>
       </c>
-      <c r="Y22" s="69" t="s">
+      <c r="Y22" s="73" t="s">
         <v>203</v>
       </c>
-      <c r="Z22" s="69"/>
-      <c r="AA22" s="69"/>
-      <c r="AB22" s="69"/>
+      <c r="Z22" s="73"/>
+      <c r="AA22" s="73"/>
+      <c r="AB22" s="73"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
@@ -9982,16 +9985,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="Y22:AB22"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="O18:W18"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="B2:AS2"/>
     <mergeCell ref="Y18:AS18"/>
     <mergeCell ref="Y13:AA13"/>
     <mergeCell ref="Y14:AA14"/>
     <mergeCell ref="Y15:AA15"/>
-    <mergeCell ref="Y22:AB22"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="O18:W18"/>
-    <mergeCell ref="B3:I3"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10422,6 +10425,9 @@
       <c r="B48" s="58" t="s">
         <v>95</v>
       </c>
+      <c r="G48" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B49" s="60" t="s">

</xml_diff>